<commit_message>
CheckoutPage and CheckoutTests (still failing
</commit_message>
<xml_diff>
--- a/TestSelenium/src/test/resources/test-data.xlsx
+++ b/TestSelenium/src/test/resources/test-data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Year 4\Software Testing and Quality Assurance\Assignment_2\TestSelenium\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE6A712C-0529-4A9A-8D81-A7D99F96FED6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5FD6137-0D6C-42F3-87AE-94DCA07ABB5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-113" yWindow="-113" windowWidth="24267" windowHeight="13023" xr2:uid="{763D8013-566B-4590-9641-73BF4B3B78CF}"/>
   </bookViews>
@@ -105,10 +105,18 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -131,13 +139,16 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -512,7 +523,7 @@
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B2" t="s">
@@ -547,7 +558,10 @@
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1" xr:uid="{336FBAD5-1DD1-44A7-8EC5-166D2880BE11}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Refactor LoginTests.java and RegistrationTests.java to read from test-data.xlsx
</commit_message>
<xml_diff>
--- a/TestSelenium/src/test/resources/test-data.xlsx
+++ b/TestSelenium/src/test/resources/test-data.xlsx
@@ -8,12 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Year 4\Software Testing and Quality Assurance\Assignment_2\TestSelenium\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5FD6137-0D6C-42F3-87AE-94DCA07ABB5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C7ACD11-763C-48EC-845E-260012C0EE9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-113" yWindow="-113" windowWidth="24267" windowHeight="13023" xr2:uid="{763D8013-566B-4590-9641-73BF4B3B78CF}"/>
+    <workbookView xWindow="1127" yWindow="1127" windowWidth="18031" windowHeight="9304" activeTab="1" xr2:uid="{763D8013-566B-4590-9641-73BF4B3B78CF}"/>
   </bookViews>
   <sheets>
     <sheet name="CheckoutProcess" sheetId="1" r:id="rId1"/>
+    <sheet name="ValidLogin" sheetId="2" r:id="rId2"/>
+    <sheet name="InvalidLogin" sheetId="3" r:id="rId3"/>
+    <sheet name="ValidRegistration" sheetId="4" r:id="rId4"/>
+    <sheet name="RegistrationValidationErrors" sheetId="5" r:id="rId5"/>
+    <sheet name="Sheet1" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="39">
   <si>
     <t>alice05@example.com</t>
   </si>
@@ -99,6 +104,63 @@
   </si>
   <si>
     <t>comment</t>
+  </si>
+  <si>
+    <t>expectedTitle</t>
+  </si>
+  <si>
+    <t>expectedLogoutVisible</t>
+  </si>
+  <si>
+    <t>My Account</t>
+  </si>
+  <si>
+    <t>expectedErrorMessage</t>
+  </si>
+  <si>
+    <t>wrongpassword</t>
+  </si>
+  <si>
+    <t>Warning: No match for E-Mail Address and/or Password.</t>
+  </si>
+  <si>
+    <t>Account Login</t>
+  </si>
+  <si>
+    <t>telephone</t>
+  </si>
+  <si>
+    <t>confirmPassword</t>
+  </si>
+  <si>
+    <t>expectedSuccessMessage</t>
+  </si>
+  <si>
+    <t>Your Account Has Been Created!</t>
+  </si>
+  <si>
+    <t>expectedEmailError</t>
+  </si>
+  <si>
+    <t>expectedTelephoneError</t>
+  </si>
+  <si>
+    <t>expectedPasswordError</t>
+  </si>
+  <si>
+    <t>Emily</t>
+  </si>
+  <si>
+    <t>E-Mail Address does not appear to be valid!</t>
+  </si>
+  <si>
+    <t>Telephone must be between 3 and 32 characters!</t>
+  </si>
+  <si>
+    <t>Password must be between 4 and 20 characters!</t>
+  </si>
+  <si>
+    <t>valid@example.com</t>
   </si>
 </sst>
 </file>
@@ -564,4 +626,224 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{139FB9E0-6030-4276-AB03-32C7C3F57A3E}">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="15.05" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CCF61071-164B-4D5E-8FB9-E817E0AA8500}">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="15.05" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68F3E6B5-4091-4ACD-A23A-514BA22AC00F}">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="15.05" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2">
+        <v>1234567890</v>
+      </c>
+      <c r="D2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{173CFE6C-6D3F-42F9-A049-18F4FF8389F3}">
+  <dimension ref="A1:I3"/>
+  <sheetFormatPr defaultRowHeight="15.05" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="3" max="3" width="17.44140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F1" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1" t="s">
+        <v>31</v>
+      </c>
+      <c r="H1" t="s">
+        <v>32</v>
+      </c>
+      <c r="I1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B2" t="s">
+        <v>1</v>
+      </c>
+      <c r="G2" t="s">
+        <v>35</v>
+      </c>
+      <c r="H2" t="s">
+        <v>36</v>
+      </c>
+      <c r="I2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D3">
+        <v>1234567890</v>
+      </c>
+      <c r="E3">
+        <v>123</v>
+      </c>
+      <c r="F3">
+        <v>123</v>
+      </c>
+      <c r="I3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A2F7B43-8B32-47F2-8F1B-0BB4E7B015FD}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.05" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>